<commit_message>
Release ReceiptLedger v1.4.1: clearer monthly charts and parallel reading
</commit_message>
<xml_diff>
--- a/templates/レシート家計簿_テンプレート.xlsx
+++ b/templates/レシート家計簿_テンプレート.xlsx
@@ -16,7 +16,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'支出一覧'!$A$1:$M$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'明細'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'月別集計'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'月別集計'!$9:$9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'月別集計'!$B$2:$L$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,11 +25,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0&quot;円&quot;;[Red]-#,##0&quot;円&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot;件&quot;"/>
+    <numFmt numFmtId="166" formatCode="0&quot;か月&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,12 +47,12 @@
       <name val="Yu Gothic"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="17"/>
+      <sz val="20"/>
     </font>
     <font>
       <name val="Yu Gothic"/>
       <color rgb="00647D8F"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Yu Gothic"/>
@@ -62,7 +64,13 @@
       <name val="Yu Gothic"/>
       <b val="1"/>
       <color rgb="0017698A"/>
-      <sz val="20"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <b val="1"/>
+      <color rgb="0017698A"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Yu Gothic"/>
@@ -72,12 +80,29 @@
     </font>
     <font>
       <name val="Yu Gothic"/>
+      <color rgb="00647D8F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="17"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <b val="1"/>
+      <color rgb="0017698A"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
       <b val="1"/>
       <color rgb="0017324A"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +119,11 @@
         <fgColor rgb="00EAF3F8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017698A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -107,33 +137,57 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -873,43 +927,176 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="008CB2A4"/>
+    <tabColor rgb="003E9A87"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="B2:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+    <row r="2" ht="42" customHeight="1">
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>月別集計 ｜ 支出の推移と内訳</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>金額は税込・費目はレシート単位。— は0円です。アプリで「Excelを保存」すると更新します。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>累計支出（税込）</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>レシート件数</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>記録のある月</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="B6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="5" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>月ごとの支出</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>費目別の内訳</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>年月</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
-        <is>
-          <t>費目</t>
-        </is>
-      </c>
-      <c r="C1" s="10" t="inlineStr">
-        <is>
-          <t>支出合計</t>
-        </is>
-      </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>税込合計</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>件数</t>
         </is>
       </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>食費</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>日用品</t>
+        </is>
+      </c>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>交通</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>医療</t>
+        </is>
+      </c>
+      <c r="I9" s="18" t="inlineStr">
+        <is>
+          <t>娯楽</t>
+        </is>
+      </c>
+      <c r="J9" s="18" t="inlineStr">
+        <is>
+          <t>住居</t>
+        </is>
+      </c>
+      <c r="K9" s="18" t="inlineStr">
+        <is>
+          <t>光熱費</t>
+        </is>
+      </c>
+      <c r="L9" s="18" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="35" customHeight="1">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>レシートを記録すると、ここに月ごとの支出とグラフが表示されます。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <mergeCells count="11">
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B3:L3"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="B10:L10"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="E8:L8"/>
+    <mergeCell ref="I5:L5"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>